<commit_message>
Đạt. Test3_fixBG.py và Arduinocode
</commit_message>
<xml_diff>
--- a/Công việc.xlsx
+++ b/Công việc.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Cài đặt Python 3.14</t>
   </si>
@@ -77,6 +77,12 @@
   </si>
   <si>
     <t>Fig lag do COM, nhưng bị spam data xuốn COM</t>
+  </si>
+  <si>
+    <t>Test3_fixBG.py vs Arduino</t>
+  </si>
+  <si>
+    <t>Test OK</t>
   </si>
 </sst>
 </file>
@@ -552,8 +558,12 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
+      <c r="B9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>

</xml_diff>